<commit_message>
Making robust changes before Scaler data upsert)
</commit_message>
<xml_diff>
--- a/benchmarking/Medical Documents Test Suit/RAG Benchmarking.xlsx
+++ b/benchmarking/Medical Documents Test Suit/RAG Benchmarking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAGner\benchmarking\Medical Documents Test Suit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98D717E8-60EB-4599-9A42-D6FBAA468B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9A9B07B-6883-499F-9207-5C2658D8A2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11235" xr2:uid="{8EE469B7-ACF9-4303-BE78-446932B45CFD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8EE469B7-ACF9-4303-BE78-446932B45CFD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
   <si>
     <t>Question</t>
   </si>
@@ -121,6 +121,39 @@
   </si>
   <si>
     <t>Method Used</t>
+  </si>
+  <si>
+    <t>Error code 5201; the most likely cause is that measurements are already in process, possibly a second instance of the ARTSENS PWV application running on the same PC. [0_artsens_manual.pdf, Page 22]</t>
+  </si>
+  <si>
+    <t>Here's a thinking process: 1. **Analyze User Question**: The user is asking about specific challenges that complicate CAD assessment in CKD patients using traditional biomarkers and imaging, and why multidisciplinary team management is essential for cardiovascular complications in this population. They want an answer based strictly on the provided context. 2. **Scan Context for Relevant Information**: I need to find passages that discuss: - Challenges in assessing CAD in CKD patients (traditional biomarkers, imaging) - Why multidisciplinary team management is essential Let me go through the excerpts: Excerpt 1 (Page 1): Mentions CKD patients excluded from CVD trials, poor generalizability, underrepresentation. Mentions CKD-related risk factors: "Non-traditional risk factors e.g. uraemia, anaemia, inflammation, oxidative stress, diabetes arterial/valvular calcification, dialysis-related factors". Also mentions "Traditional risk factors e.g. hypertension". Mentions mortality increases with CKD progression. But doesn't specifically detail challenges with traditional biomarkers/img for CAD assessment. Excerpt 2 (Page 3): Discusses multidisciplinary approach, complex bidirectional relationship, common multimorbidity, limitations of standardized risk scores, benefit from corroboration between specialists. Mentions "Standardised risk scores that are often used to guide investigations and management in CVD are likely to underestimate risk in CKD". This is relevant to the "why multidisciplinary is essential" part, and touches on risk score limitations. Excerpt 3 (Page 4): Mentions complexity, need for multidisciplinary approach, but no specific details on biomarkers/img challenges. Excerpt 4 (Page 1): Has Figure 1 description: "Changing Cardiovascular Disease Risk in Progressing Chronic Kidney Disease". Shows non-atherosclerotic CVD events (LVH, arrhythmias, SCD, haemorrhagic stroke) and atherosclerotic CVD events (AMI, ischaemic stroke, PAD). Notes: "As CKD progresses, the risk of CVD events rises. Mortality following cardiovascular events also increases. Non-atherosclerotic causes contribute more than atherosclerotic causes as CKD progresses". Also mentions: "Traditional risk factors e.g. hypertension... Non-traditional risk factors e.g. uraemia, anaemia, inflammation, oxidative stress, diabetes arterial/valvular calcification, dialysis-related factors". This implies traditional risk factors may not fully capture CVD risk in CKD, and non-traditional factors become more dominant. Excerpt 5 (Page 1): Mentions current treatment options associated with high burden of adverse events, concerns about dose adjustments for renally-excreted medications, clinicians act with caution, CVD being under-treated. Also mentions the article focuses on CAD, arrhythmias, HF, VHD. Now, I need to synthesize an answer that directly addresses: - Specific challenges complicating CAD assessment using traditional biomarkers and imaging in CKD - Why multidisciplinary team management is essential Let me extract precise points from context: From Excerpt 4 (Page 1): The figure shows that as CKD progresses, non-atherosclerotic CVD events (LVH, arrhythmias, SCD, haemorrhagic stroke) become more prominent alongside atherosclerotic events (AMI, ischaemic stroke, PAD). It lists "Traditional risk factors e.g. hypertension" and "Non-traditional risk factors e.g. uraemia, anaemia, inflammation, oxidative stress, diabetes arterial/valvular calcification, dialysis-related factors". This suggests traditional risk factors (like hypertension, diabetes) may not adequately predict CAD in CKD because non-traditional factors (uraemia, anaemia, inflammation, oxidative stress, vascular calcification, dialysis-related factors) increasingly contribute to CVD risk and may confound or obscure traditional biomarker-based assessment. From Excerpt 2 (Page 3): "Standardised risk scores that are often used to guide investigations and management in CVD are likely to underestimate risk in CKD." This directly addresses challenges with traditional risk assessment tools/biomarkers. From Excerpt 2 (Page 3) also: "The complex bidirectional relationship between CVD and CKD, combined with common multimorbidity and limitations of standardised risk scores, benefit from corroboration between specialists. A multidisciplinary team approach including cardiologist, nephrologists and allied healthcare professionals improves management and patient-centred HF care through joint clinics." This explains why multidisciplinary management is essential: due to complexity, bidirectional relationship, multimorbidity, and limitations of standardized risk scores. From Excerpt 1 (Page 1): "CKD patients are largely excluded from clinical studies, resulting in a poor generalisability of assessment tools and a poor evidence base for the safety and efficacy of available treatments." This adds context about why assessment tools lack generalizability. From Excerpt 5 (Page 1): "current treatment options are associated with a high burden of adverse events, complications and concerns about dose adjustments particularly for renally-excreted medications.</t>
+  </si>
+  <si>
+    <t>Here's a thinking process: 1. **Analyze User Question**: The user is asking for the recommended blood pressure target for adults with confirmed hypertension and a 10-year ASCVD event risk of 10% or higher, according to the 2019 ACC/AHA Guideline on Primary Prevention. 2. **Scan Context for Relevant Information**: I need to find where blood pressure targets or recommendations for hypertension with ASCVD risk are mentioned. Let me look through the provided context. - Data Table 1 (Page 21): Has recommendations about BP-lowering medication for adults with estimated 10-year ASCVD risk &lt;10% and SBP ≥140 or DBP ≥90. It says: "In adults with an estimated 10-year ASCVD risk &lt;10% and an SBP of 140 mm Hg or higher or a DBP of 90 mm Hg or higher, initiation and use of BP-lowering medication are recommended." But this is for risk &lt;10%, not ≥10%. - Data Table 3 (Page 17): About cholesterol/statin therapy, not BP targets. - Document Excerpt 2 (Page 21): Mentions hypertension prevalence, definitions (SBP ≥130 or DBP ≥80), and risk associations, but not specific treatment targets for risk ≥10%. - Document Excerpt 4 (Page 10): About lifetime/30-year risk estimation, not BP targets. - Document Excerpt 5 (Page 8): About screening risk factors, PCE, etc. Wait, let me re-read carefully. The question asks: "what is the recommended blood pressure target for adults with confirmed hypertension and a 10-year ASCVD event risk of 10% or higher?" Looking at Data Table 1, Page 21: The row mentions "I C-LD 6. In adults with an estimated 10-year ASCVD risk &lt;10% and an SBP of 140 mm Hg or higher or a DBP of 90 mm Hg or higher, initiation and use of BP-lowering medication are recommended." This is for risk &lt;10%. What about risk ≥10%? The table might have other rows, but only one row is shown partially. The text says: "| | 7. In adults with confirmed hypertension without additional markers of increased ..." and then it cuts off. Actually, the table data shows: "| | | Recommendations | | --- | --- | --- | | I | C-LD | 6. In adults with an estimated 10-year ASCVD risk &lt;10% and an SBP of 140 mm Hg or higher or a DBP of 90 mm Hg or higher, initiation and use of BP-lowering medication are recommended.54:436:54:4-55-$4.4-58 Adapted from recommendations in the 2017 Hypertension Clinical Practice Guidelines.\*4\*" | | | 7. In adults with confirmed hypertension without additional markers of increased |" So row 7 is cut off. But the question is about risk ≥10% or specifically 10% or higher. The table explicitly mentions risk &lt;10%. I need to check if there's a recommendation for risk ≥10% elsewhere. Let me search the context for "10-year ASCVD risk" and "hypertension" and "blood pressure target". From Document Excerpt 2: "The prevalence of hypertension (defined as systolic blood pressure [SBP] ≥130 mm Hg or diastolic blood pressure [DBP] ≥80 mm Hg) among US adults is 46%..." This defines hypertension, but not treatment targets per risk category. Data Table 1 seems to have a row 7 that's incomplete: "7. In adults with confirmed hypertension without additional markers of increased ..." It might continue with something about risk ≥10% or different BP targets. Wait, the context says: "--- Data Table 1 (Source: ..., Page: 21) --- **Context preceding table:** ... **Table Data:** | | | Recommendations | | --- | --- | --- | | I | C-LD | 6. In adults with an estimated 10-year ASCVD risk &lt;10% and an SBP of 140 mm Hg or higher or a DBP of 90 mm Hg or higher, initiation and use of BP-lowering medication are recommended.54:436:54:4-55-$4.4-58 Adapted from recommendations in the 2017 Hypertension Clinical Practice Guidelines.\*4</t>
+  </si>
+  <si>
+    <t>According to the 2018 Guidelines for the Management of Dyslipidemia, the four major modifiable CVD risk factors in Korean men are hypertension, smoking, dyslipidemia, and diabetes. Their combined population attributable risk reaches 64% [2018 Guidelines for the management of dyslipidemia.pdf, Page 4]. [2018 Guidelines for the management of dyslipidemia.pdf, Page 4]</t>
+  </si>
+  <si>
+    <t>I cannot answer this question based on the provided documents.</t>
+  </si>
+  <si>
+    <t>According to the SphygmoCor XCEL Operators Manual, the specific troubleshooting steps for Error Code 87 (Unable to continue Brachial Assessment due to inflate timeout) are: 1. Ensure that the hose connections to the device and cuff are intact and tight. 2. Ensure use of correct cuff size, correct positioning and fit. 3. Ensure that the cuff is not leaking air. 4. After completing the above steps, attempt another measurement. [R4] SphygmoCor XCEL Operators Manual.pdf, Page 88</t>
+  </si>
+  <si>
+    <t>Based on the provided context, I can identify the LDL-C target levels for four of the five cardiovascular risk categories, but the "extremely high risk" category is not explicitly defined in the documents. Here are the findings: **Low-risk group**: LDL-C target is &lt; 160 mg/dL. Statin therapy may be used if LDL-C is ≥ 160 mg/dL. Patients with one or fewer major risk factors other than LDL-C are classified as the low-risk group (Source: 2018 Guidelines for the management of dyslipidemia.pdf, Page 12 and Page 22). **Moderate-risk group**: LDL-C target is &lt; 130 mg/dL. Statin therapy should be started when LDL-C is ≥ 130 mg/dL but could be started even for those with LDL-C level 100 to 129 mg/dL when patients have multiple CV risk factors. This group includes patients with two or more CV risk factors (Source: 2018 Guidelines for the management of dyslipidemia.pdf, Page 22). **High-risk group**: LDL-C target is &lt; 100 mg/dL. Statin treatment should be started if LDL-C is ≥ 100 mg/dL, and could be selectively considered even for patients with an LDL-C level of &lt; 100 mg/dL (Source: 2018 Guidelines for the management of dyslipidemia.pdf, Page 22). **Very high-risk group**: LDL-C target is &lt; 70 mg/dL or by more than 50% of the baseline level. This group includes patients with CVD (CAD, peripheral artery disease, ischemic stroke, transient ischemic attack) (Source: 2018 Guidelines for the management of dyslipidemia.pdf, Page 8 and Page 22). **Extremely high-risk group**: The provided documents do not define an "extremely high risk" category or specify exact LDL-C targets for this group. The documents only mention "very high-risk group" and "high-risk group" but do not use the term "extremely high risk" or provide information about which patient populations would fall into this category. I cannot answer this question based on the provided documents.</t>
+  </si>
+  <si>
+    <t>Based on the provided context, the CKD-specific non-traditional risk factors that significantly contribute to cardiovascular disease include: **Non-Traditional Risk Factors:** 1. Uraemia 2. Anaemia 3. Inflammation 4. Oxidative stress 5. Arterial/valvular calcification 6. Dialysis-related factors [Cardiovascular Complications of Chronic Kidney Disease.pdf, Page 1] **Mechanistic Increase in CVD Risk:** These CKD-related factors contribute more significantly as estimated glomerular filtration rate (eGFR) declines. The mechanism by which they increase CVD risk is reflected in the changing pathophysiology of CVD in CKD patients—specifically, non-atherosclerotic cardiac events become increasingly common as CKD progresses. Unlike traditional risk factors that primarily drive atherosclerotic events (such as acute MI, ischaemic stroke, and peripheral arterial disease), these non-traditional factors predominantly contribute to non-atherosclerotic CVD events including left ventricular hypertrophy (LVH), arrhythmias, sudden cardiac death (SCD), and haemorrhagic stroke. Additionally, time is an important mechanistic factor—the longer time spent in each stage of CKD before commencing dialysis results in longer exposure to these risk factors, leading to greater accumulated damage and increased CVD risk. [Cardiovascular Complications of Chronic Kidney Disease.pdf, Page 1]</t>
+  </si>
+  <si>
+    <t>Based on the provided context, the specific reuse life limits for the ARTSENS Plus PWV device probe and cuff are as follows: **Cuff** [0_artsens_manual.pdf, Page 20]: - The cuff's reuse life is defined by the manufacturer at **10,000 cycles of operation**. - The **Velcro tapes** of the cuff must withstand a minimum of **1,000 open-close cycles** without failure. - The **Cuff Bladder** is capable of enduring at least **10,000 pressure cycles** inflated to **300 mmHg** without compromising functionality. **Probe** [0_artsens_manual.pdf, Page 20]: - The lifespan for the probe is **5 years**. - The reuse life extends until the probe either fails during the self-test procedure or exhibits visible physical damage on its cables.</t>
+  </si>
+  <si>
+    <t>The model failed to generate a response. It may have encountered an internal error or triggered a content filter on the provider's end.</t>
+  </si>
+  <si>
+    <t>Based on the provided context, when using the Artsens Plus PWV device: **Method for Measuring PWV Distance:** - Measure the PWV distance from the carotid site on the left side of the neck to the top of the thigh cuff - The measurement must be taken above the patient's body using the Carotid Site and the Top of Thigh Cuff as landmarks - The measurement is taken in a straight line above the body (not following body contours) - Using the centimetre scale on the measuring tape, measure the PWV distance, then divide by 10 to convert to millimetres and enter into the software - The device calculates the direct method distance as 80% of the Carotid-to-Thigh cuff distance **Why It Must Not Follow Body Contours:** "The PWV distance should not use patient contact where the individual contours of the patients' body can incorrectly increase PWV distance based on their own individual anatomical external body structure." This ensures accurate and consistent measurements by avoiding artificial inflation of the distance measurement that would result from following the individual anatomical variations of each patient's body shape. **Sources:** - [0_artsens_manual.pdf, Page 15] - [0_artsens_manual.pdf, Multiple Pages (Summary)]</t>
   </si>
 </sst>
 </file>
@@ -474,6 +507,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6796CB8-0435-4506-8BE0-271492F21DDB}">
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="22" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -499,6 +535,9 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
+      <c r="C2" t="s">
+        <v>32</v>
+      </c>
       <c r="E2" t="s">
         <v>25</v>
       </c>
@@ -510,6 +549,9 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
       <c r="E3" t="s">
         <v>26</v>
       </c>
@@ -521,6 +563,9 @@
       <c r="B4" t="s">
         <v>7</v>
       </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
       <c r="E4" t="s">
         <v>27</v>
       </c>
@@ -532,6 +577,9 @@
       <c r="B5" t="s">
         <v>9</v>
       </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
       <c r="E5" t="s">
         <v>28</v>
       </c>
@@ -543,6 +591,9 @@
       <c r="B6" t="s">
         <v>11</v>
       </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
       <c r="E6" t="s">
         <v>27</v>
       </c>
@@ -554,6 +605,9 @@
       <c r="B7" t="s">
         <v>13</v>
       </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
       <c r="E7" t="s">
         <v>29</v>
       </c>
@@ -565,6 +619,9 @@
       <c r="B8" t="s">
         <v>15</v>
       </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
       <c r="E8" t="s">
         <v>27</v>
       </c>
@@ -576,6 +633,9 @@
       <c r="B9" t="s">
         <v>17</v>
       </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
       <c r="E9" t="s">
         <v>26</v>
       </c>
@@ -587,6 +647,9 @@
       <c r="B10" t="s">
         <v>19</v>
       </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
       <c r="E10" t="s">
         <v>28</v>
       </c>
@@ -598,6 +661,9 @@
       <c r="B11" t="s">
         <v>21</v>
       </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
       <c r="E11" t="s">
         <v>25</v>
       </c>
@@ -608,6 +674,9 @@
       </c>
       <c r="B12" t="s">
         <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>

</xml_diff>